<commit_message>
P-2026-0046 REV. 1: Actualizar con bastidor simple T50, sin galvanizar, coste ullastre 200 y cables inox
</commit_message>
<xml_diff>
--- a/presupuestos/P-2026-0046-pergola-rustica-ullastre-metal-canizo-binibeca/presupuesto.xlsx
+++ b/presupuestos/P-2026-0046-pergola-rustica-ullastre-metal-canizo-binibeca/presupuesto.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P-2026-0046 Pergola Ullastre" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P-2026-0046 Ullastre T50" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -516,7 +516,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PRESUPUESTO TÉCNICO Y VALORACIÓN ECONÓMICA: P-2026-0046</t>
+          <t>PRESUPUESTO TÉCNICO Y VALORACIÓN ECONÓMICA: P-2026-0046 (REV. 1)</t>
         </is>
       </c>
     </row>
@@ -576,7 +576,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Pérgola rústica de madera de Ullastre y metal termolacado con cubierta de cañizo y anclajes ocultos para pies descalzos</t>
+          <t>Pérgola rústica de madera de Ullastre y bastidor metálico en simple T de 50 mm con cubierta de cañizo, entramado tensor inox y anclajes ocultos para pies descalzos</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Medidas: 4,00 x 3,00 x 2,50 m (12 m²) | Troncos de Ullastre Ø140-180 mm | Bastidor acero 100x50x3 y 50x30x2 mm S275JR | Acabado Dúplex C5-M Marino (Galvanizado en caliente + Poliéster al horno) | Cables tensores Inox AISI 316 para trepadoras | Cañizo natural cosido | Casquillos empotrados Inox 316 (cero resaltes para transitar descalzo)</t>
+          <t>Medidas: 4,00 x 3,00 x 2,50 m (12 m²) | 3 troncos de Ullastre autóctono de Menorca (coste HAM 200€/ud) | Bastidor ligero en perfil simple T de 50 mm (T 50x50x5 S275JR) para alojamiento exacto de cañizo | Acabado exterior pintado (sin galvanizar): imprimación epoxi + poliuretano | Entramado tensor de cables Inox AISI 316 para trepadoras | Cañizo natural cosido | Casquillos empotrados Inox 316 (cero resaltes para transitar descalzo)</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="12" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="F13" s="12">
         <f>D13*E13</f>
@@ -671,7 +671,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="12" t="n">
-        <v>560</v>
+        <v>480</v>
       </c>
       <c r="F14" s="12">
         <f>D14*E14</f>
@@ -686,7 +686,7 @@
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>Pilares estructurales de madera maciza de Ullastre (acebuche) autóctono de Menorca (Ø140-180 mm, h=2,60 m): descortezado manual, lijado artesanal, saneado y doble lasur protector UV marino poro abierto; mecanizado de testas para vástagos ocultos</t>
+          <t>Pilares estructurales de madera maciza de Ullastre (acebuche) autóctono de Menorca (Ø140-180 mm, h=2,60 m, coste base HAM 200€/ud): descortezado manual, saneado y doble lasur protector UV marino poro abierto; mecanizado de testas para vástagos ocultos</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
@@ -698,7 +698,7 @@
         <v>3</v>
       </c>
       <c r="E15" s="12" t="n">
-        <v>460</v>
+        <v>340</v>
       </c>
       <c r="F15" s="12">
         <f>D15*E15</f>
@@ -713,7 +713,7 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>Fabricación en taller de bastidor metálico estructural y correas: vigas en tubo 100x50x3 mm S275JR, correas intermedias 50x30x2 mm cada 65 cm, cazoletas de apoyo en ullastre y fijaciones químicas murales inox A4</t>
+          <t>Fabricación en taller de bastidor metálico en perfil simple T de 50 mm (T 50x50x5 mm S275JR): marco perimetral y viguetas intermedias que alojan el cañizo, cazoletas ocultas sobre ullastres y anclajes químicos murales inox A4</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
@@ -725,7 +725,7 @@
         <v>1</v>
       </c>
       <c r="E16" s="12" t="n">
-        <v>1840</v>
+        <v>980</v>
       </c>
       <c r="F16" s="12">
         <f>D16*E16</f>
@@ -740,7 +740,7 @@
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>Tratamiento anticorrosivo Sistema Dúplex C5-M (Máxima durabilidad marina): Galvanizado por inmersión en caliente UNE-EN ISO 1461 (&gt;85 µm) + Termolacado al horno con polvo de poliéster texturado Qualisteelcoat</t>
+          <t>Tratamiento superficial de pintura anticorrosiva de exterior (sin galvanizar): desengrasado, limpieza mecánica, imprimación epoxi fosfatante de alto espesor y esmalte poliuretano alifático bicomponente para intemperie marina</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
@@ -752,7 +752,7 @@
         <v>1</v>
       </c>
       <c r="E17" s="12" t="n">
-        <v>640</v>
+        <v>340</v>
       </c>
       <c r="F17" s="12">
         <f>D17*E17</f>
@@ -767,7 +767,7 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>Emparrillado tensor para plantas trepadoras en Inox AISI 316: retícula de cables trenzados 1x19 Ø4mm o varillas Ø6mm cada 50 cm con tensores de botella náuticos A4 para soporte de carga vegetal y resistencia a Tramuntana</t>
+          <t>Entramado tensor de cables de acero inoxidable AISI 316 para trepadoras: retícula de cables 1x19 Ø4mm cada 50 cm con tensores de botella náuticos A4 para soporte de carga vegetal y resistencia a vientos</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
@@ -779,7 +779,7 @@
         <v>1</v>
       </c>
       <c r="E18" s="12" t="n">
-        <v>490</v>
+        <v>440</v>
       </c>
       <c r="F18" s="12">
         <f>D18*E18</f>
@@ -794,7 +794,7 @@
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>Cubierta de sombreo inmediato de cañizo natural nacional de caña entera, colocado sobre estructura y afianzado con pletinas metálicas y bridas de acero inoxidable AISI 316 cada 30 cm</t>
+          <t>Cubierta de sombreo inmediato de cañizo natural nacional de caña entera, encastrado sobre las alas de los perfiles T de 50 mm con pletinas metálicas y bridas de acero inoxidable AISI 316 cada 30 cm</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
@@ -806,7 +806,7 @@
         <v>14</v>
       </c>
       <c r="E19" s="12" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="F19" s="12">
         <f>D19*E19</f>
@@ -821,7 +821,7 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>Transporte a obra a Binibeca Vell, medios auxiliares y montaje en dos fases (Fase 1 entrega/nivelación de vainas; Fase 2 izado bastidor, aplomado ullastres, tendido de cañizo y red de trepadoras)</t>
+          <t>Transporte a obra a Binibeca Vell, medios auxiliares y montaje en dos fases (Fase 1 entrega/nivelación de vainas; Fase 2 izado bastidor T50, aplomado ullastres, encastre de cañizo y red de cables inox)</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
@@ -833,7 +833,7 @@
         <v>1</v>
       </c>
       <c r="E20" s="12" t="n">
-        <v>1150</v>
+        <v>950</v>
       </c>
       <c r="F20" s="12">
         <f>D20*E20</f>
@@ -885,7 +885,7 @@
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>5480</v>
+        <v>3950</v>
       </c>
     </row>
     <row r="27">
@@ -895,7 +895,7 @@
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>6630.8</v>
+        <v>4779.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>